<commit_message>
EP N°1 Sacyr: ajusta a cláusula 5 Facturación del contrato
Columnas a origen Anterior/Presente/Acumulado, descripciones idénticas
al Anexo 1, condiciones de aprobación y plazo de factura, y listado de
documentos de respaldo exigidos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VyQP4PFH1JMjNsbtJ3bdY5
</commit_message>
<xml_diff>
--- a/06_Estados_de_Pago/EP_N1_Sacyr_Ruta_Itata.xlsx
+++ b/06_Estados_de_Pago/EP_N1_Sacyr_Ruta_Itata.xlsx
@@ -10,7 +10,7 @@
     <sheet name="EP N°1, Rev-0" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'EP N°1, Rev-0'!$A$1:$Q$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'EP N°1, Rev-0'!$A$1:$Q$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -591,6 +591,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -969,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.44140625" customWidth="1" min="1" max="1"/>
@@ -1121,7 +1124,7 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>AVANCE (unid)</t>
+          <t>CANTIDADES (a origen)</t>
         </is>
       </c>
       <c r="I10" s="19" t="n"/>
@@ -1178,7 +1181,7 @@
       </c>
       <c r="I11" s="24" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="J11" s="24" t="inlineStr">
@@ -1193,7 +1196,7 @@
       </c>
       <c r="L11" s="24" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="M11" s="24" t="inlineStr">
@@ -1208,7 +1211,7 @@
       </c>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="P11" s="24" t="inlineStr">
@@ -1450,7 +1453,7 @@
       </c>
       <c r="B16" s="31" t="inlineStr">
         <is>
-          <t>Instalación de faena: señalética, balizas, baños y agua para perforación (incluido)</t>
+          <t>Instalación de faena: Señalética, balizas, baños y agua para perforación (incluido)</t>
         </is>
       </c>
       <c r="C16" s="32" t="inlineStr">
@@ -1877,7 +1880,7 @@
       </c>
       <c r="B23" s="31" t="inlineStr">
         <is>
-          <t>Ensayo corte directo (ASTM D3080/D3080M-11)</t>
+          <t>Ensayo corte directo (ASTM S3080/D3080M-11)</t>
         </is>
       </c>
       <c r="C23" s="32" t="inlineStr">
@@ -1944,7 +1947,7 @@
       </c>
       <c r="B24" s="31" t="inlineStr">
         <is>
-          <t>Ensayo triaxial (ASTM D7181-11) (1 probeta)</t>
+          <t>Ensayo triaxial (ASTM D7181-11) (1 PROBETA)</t>
         </is>
       </c>
       <c r="C24" s="32" t="inlineStr">
@@ -2130,84 +2133,119 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="59" t="inlineStr">
         <is>
-          <t>•  EP N°1 cobra el 100% de las partidas de sondaje en cauce (ítems 2 al 9 del Anexo 1). Los ensayes de laboratorio (ítems 11 al 13) se cobrarán en un próximo EP.</t>
+          <t>•  EP relacionado a origen (cláusula 5.3): columnas Anterior / Presente / Acumulado. EP N°1: acumulado anterior = 0.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="12" customHeight="1">
       <c r="B35" s="59" t="inlineStr">
         <is>
-          <t>•  Retención 5% por garantía según cláusula 9 (Retención por Garantía), devolutiva a los 3 meses de la firma del Finiquito.</t>
+          <t>•  Cobra el 100% de las partidas de sondaje en cauce ejecutadas (ítems 2 al 9 del Anexo 1), respaldadas con informe de sondaje y registro de metros perforados. Ensayes de laboratorio (ítems 11 al 13) no se cobran en este EP.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="12" customHeight="1">
       <c r="B36" s="59" t="inlineStr">
         <is>
-          <t>•  La factura debe indicar el N° de contrato 30803000661I000015 en referencia y glosa. Enviar a terceros-76885606@dte.iconstruye.com.</t>
+          <t>•  Solo incluye partidas del Anexo N°1 del Contrato, a precios fijos del mismo. No incluye materiales en acopio.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="B37" s="59" t="inlineStr">
         <is>
-          <t>•  Condición de pago: 30 días desde la recepción de la factura. Precios netos; IVA desglosado en factura.</t>
+          <t>•  Aprobación del Contratista en máx. 15 días desde su presentación. Aprobado el EP, se emite una única factura, a más tardar el día 10 del mes (o hábil siguiente).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="12" customHeight="1">
       <c r="B38" s="59" t="inlineStr">
         <is>
-          <t>•  Valores expresados en pesos chilenos (CLP).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="C42" s="60" t="n"/>
-      <c r="D42" s="61" t="n"/>
-      <c r="E42" s="61" t="n"/>
-      <c r="F42" s="61" t="n"/>
-      <c r="G42" s="61" t="n"/>
-      <c r="L42" s="60" t="n"/>
-      <c r="M42" s="61" t="n"/>
-      <c r="N42" s="61" t="n"/>
-      <c r="O42" s="61" t="n"/>
-      <c r="P42" s="61" t="n"/>
-      <c r="Q42" s="61" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1">
-      <c r="C43" s="62" t="inlineStr">
+          <t>•  La factura debe indicar el N° de contrato 30803000661I000015 en referencia y glosa; enviar a terceros-76885606@dte.iconstruye.com. Pago a 30 días. IVA desglosado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="B39" s="59" t="inlineStr">
+        <is>
+          <t>•  Retención 5% por garantía (cláusula 9), devolutiva a los 3 meses de la firma del Finiquito. Valores en CLP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="12" customHeight="1">
+      <c r="B40" s="60" t="inlineStr">
+        <is>
+          <t>DOCUMENTOS QUE ACOMPAÑAN LA FACTURA (cláusula 5, N°5):</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="B41" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   5.1 EP aprobado y firmado por Sacyr  ·  5.2 Comprobante pago IVA (F29) del mes anterior  ·  5.3 Certificado F30-1 de la Inspección del Trabajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="12" customHeight="1">
+      <c r="B42" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   5.4 Nómina de trabajadores, contratos, liquidaciones, planillas de cotizaciones pagadas y finiquitos (si aplica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="12" customHeight="1">
+      <c r="B43" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   5.5 Declaración jurada simple de pago a subcontratistas y proveedores (con listado)  ·  5.6 Factura  ·  5.7 Copia firmada del Contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="61" t="n"/>
+      <c r="D47" s="62" t="n"/>
+      <c r="E47" s="62" t="n"/>
+      <c r="F47" s="62" t="n"/>
+      <c r="G47" s="62" t="n"/>
+      <c r="L47" s="61" t="n"/>
+      <c r="M47" s="62" t="n"/>
+      <c r="N47" s="62" t="n"/>
+      <c r="O47" s="62" t="n"/>
+      <c r="P47" s="62" t="n"/>
+      <c r="Q47" s="62" t="n"/>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="C48" s="63" t="inlineStr">
         <is>
           <t>Representante Contratista</t>
         </is>
       </c>
-      <c r="L43" s="62" t="inlineStr">
+      <c r="L48" s="63" t="inlineStr">
         <is>
           <t>p. SOLUT Ingeniería SpA</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
-      <c r="C44" s="63" t="inlineStr">
+    <row r="49" ht="15" customHeight="1">
+      <c r="C49" s="64" t="inlineStr">
         <is>
           <t>Sacyr Asesorías y Diseño SpA</t>
         </is>
       </c>
-      <c r="L44" s="63" t="inlineStr">
+      <c r="L49" s="64" t="inlineStr">
         <is>
           <t>Felipe Matamala Andrades — Ingeniero Civil</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="L45" s="63" t="inlineStr">
+    <row r="50" ht="15" customHeight="1">
+      <c r="L50" s="64" t="inlineStr">
         <is>
           <t>RUT: 77.625.106-2</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="64" t="inlineStr">
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="65" t="inlineStr">
         <is>
           <t>Maipu 1623 – Concepción – Fonos: +56 9 3006 2244 – fmatamala@solut.cl – www.solut.cl</t>
         </is>
@@ -2215,11 +2253,9 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C49:G49"/>
     <mergeCell ref="N2:P2"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="L42:Q42"/>
     <mergeCell ref="I27:J27"/>
-    <mergeCell ref="L45:Q45"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="N29:P29"/>
     <mergeCell ref="A6:Q6"/>
@@ -2228,20 +2264,22 @@
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="K27:M27"/>
     <mergeCell ref="N28:P28"/>
+    <mergeCell ref="C47:G47"/>
     <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="C44:G44"/>
-    <mergeCell ref="L44:Q44"/>
+    <mergeCell ref="L50:Q50"/>
     <mergeCell ref="N31:P31"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C43:G43"/>
     <mergeCell ref="K10:M10"/>
+    <mergeCell ref="L49:Q49"/>
     <mergeCell ref="O27:P27"/>
-    <mergeCell ref="A47:Q47"/>
+    <mergeCell ref="L48:Q48"/>
     <mergeCell ref="A5:Q5"/>
+    <mergeCell ref="C48:G48"/>
     <mergeCell ref="A8:Q8"/>
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="A4:Q4"/>
-    <mergeCell ref="L43:Q43"/>
+    <mergeCell ref="A52:Q52"/>
+    <mergeCell ref="L47:Q47"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>